<commit_message>
Add daily title recommendations for 2026-09-22
</commit_message>
<xml_diff>
--- a/data/output/微信24h热文榜_题目库_截至20260922.xlsx
+++ b/data/output/微信24h热文榜_题目库_截至20260922.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R5022c06c28334cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始题目库" sheetId="2" r:id="Rfaf94a1b3a004147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熟龄题目分析" sheetId="3" r:id="R6395eee484e64f4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="母题库" sheetId="4" r:id="R95fcc552599c4162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日选题" sheetId="5" r:id="R2f99c9521de04607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R704390f553784e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始题目库" sheetId="2" r:id="R62f2755b55374d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熟龄题目分析" sheetId="3" r:id="Rc60b8245dba2400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="母题库" sheetId="4" r:id="R3709e65f6ab14f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日选题" sheetId="5" r:id="R422677ac52194f69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -279,29 +279,29 @@
     <x:tableColumn id="1" name="rank"/>
     <x:tableColumn id="2" name="level"/>
     <x:tableColumn id="3" name="selection_reason"/>
-    <x:tableColumn id="4" name="topic_id"/>
-    <x:tableColumn id="5" name="first_seen_date"/>
-    <x:tableColumn id="6" name="latest_seen_date"/>
-    <x:tableColumn id="7" name="appearance_count"/>
-    <x:tableColumn id="8" name="max_heat"/>
-    <x:tableColumn id="9" name="latest_heat"/>
-    <x:tableColumn id="10" name="title"/>
-    <x:tableColumn id="11" name="description"/>
-    <x:tableColumn id="12" name="publish_time"/>
-    <x:tableColumn id="13" name="link"/>
-    <x:tableColumn id="14" name="thumbnail"/>
-    <x:tableColumn id="15" name="series"/>
-    <x:tableColumn id="16" name="category"/>
-    <x:tableColumn id="17" name="mother_topic"/>
-    <x:tableColumn id="18" name="mature_fit"/>
-    <x:tableColumn id="19" name="audience_age"/>
-    <x:tableColumn id="20" name="gender_tendency"/>
-    <x:tableColumn id="21" name="emotion"/>
-    <x:tableColumn id="22" name="need"/>
-    <x:tableColumn id="23" name="title_skeleton"/>
-    <x:tableColumn id="24" name="source_files"/>
-    <x:tableColumn id="25" name="duplicate_status"/>
-    <x:tableColumn id="26" name="data_note"/>
+    <x:tableColumn id="4" name="recommended_title"/>
+    <x:tableColumn id="5" name="topic_id"/>
+    <x:tableColumn id="6" name="first_seen_date"/>
+    <x:tableColumn id="7" name="latest_seen_date"/>
+    <x:tableColumn id="8" name="appearance_count"/>
+    <x:tableColumn id="9" name="max_heat"/>
+    <x:tableColumn id="10" name="latest_heat"/>
+    <x:tableColumn id="11" name="title"/>
+    <x:tableColumn id="12" name="description"/>
+    <x:tableColumn id="13" name="publish_time"/>
+    <x:tableColumn id="14" name="link"/>
+    <x:tableColumn id="15" name="thumbnail"/>
+    <x:tableColumn id="16" name="series"/>
+    <x:tableColumn id="17" name="category"/>
+    <x:tableColumn id="18" name="mother_topic"/>
+    <x:tableColumn id="19" name="mature_fit"/>
+    <x:tableColumn id="20" name="audience_age"/>
+    <x:tableColumn id="21" name="gender_tendency"/>
+    <x:tableColumn id="22" name="emotion"/>
+    <x:tableColumn id="23" name="need"/>
+    <x:tableColumn id="24" name="title_skeleton"/>
+    <x:tableColumn id="25" name="source_files"/>
+    <x:tableColumn id="26" name="duplicate_status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -31511,7 +31511,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90aae93e61d4c7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64bd5c05afe74f41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40187,7 +40187,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12df9d00e0a843d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e4375134fac490f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40579,7 +40579,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ba116a43b3f403a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f16b54dbe8e47c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40591,30 +40591,31 @@
     <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="42" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="12" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="14" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="14" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="14" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="12" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="14" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="12" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="18" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -40686,75 +40687,78 @@
         <x:v>selection_reason</x:v>
       </x:c>
       <x:c r="D3" s="33" t="str">
+        <x:v>recommended_title</x:v>
+      </x:c>
+      <x:c r="E3" s="33" t="str">
         <x:v>topic_id</x:v>
       </x:c>
-      <x:c r="E3" s="33" t="str">
+      <x:c r="F3" s="33" t="str">
         <x:v>first_seen_date</x:v>
       </x:c>
-      <x:c r="F3" s="33" t="str">
+      <x:c r="G3" s="33" t="str">
         <x:v>latest_seen_date</x:v>
       </x:c>
-      <x:c r="G3" s="33" t="str">
+      <x:c r="H3" s="33" t="str">
         <x:v>appearance_count</x:v>
       </x:c>
-      <x:c r="H3" s="33" t="str">
+      <x:c r="I3" s="33" t="str">
         <x:v>max_heat</x:v>
       </x:c>
-      <x:c r="I3" s="33" t="str">
+      <x:c r="J3" s="33" t="str">
         <x:v>latest_heat</x:v>
       </x:c>
-      <x:c r="J3" s="33" t="str">
+      <x:c r="K3" s="33" t="str">
         <x:v>title</x:v>
       </x:c>
-      <x:c r="K3" s="33" t="str">
+      <x:c r="L3" s="33" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="L3" s="33" t="str">
+      <x:c r="M3" s="33" t="str">
         <x:v>publish_time</x:v>
       </x:c>
-      <x:c r="M3" s="33" t="str">
+      <x:c r="N3" s="33" t="str">
         <x:v>link</x:v>
       </x:c>
-      <x:c r="N3" s="33" t="str">
+      <x:c r="O3" s="33" t="str">
         <x:v>thumbnail</x:v>
       </x:c>
-      <x:c r="O3" s="33" t="str">
+      <x:c r="P3" s="33" t="str">
         <x:v>series</x:v>
       </x:c>
-      <x:c r="P3" s="33" t="str">
+      <x:c r="Q3" s="33" t="str">
         <x:v>category</x:v>
       </x:c>
-      <x:c r="Q3" s="33" t="str">
+      <x:c r="R3" s="33" t="str">
         <x:v>mother_topic</x:v>
       </x:c>
-      <x:c r="R3" s="33" t="str">
+      <x:c r="S3" s="33" t="str">
         <x:v>mature_fit</x:v>
       </x:c>
-      <x:c r="S3" s="33" t="str">
+      <x:c r="T3" s="33" t="str">
         <x:v>audience_age</x:v>
       </x:c>
-      <x:c r="T3" s="33" t="str">
+      <x:c r="U3" s="33" t="str">
         <x:v>gender_tendency</x:v>
       </x:c>
-      <x:c r="U3" s="33" t="str">
+      <x:c r="V3" s="33" t="str">
         <x:v>emotion</x:v>
       </x:c>
-      <x:c r="V3" s="33" t="str">
+      <x:c r="W3" s="33" t="str">
         <x:v>need</x:v>
       </x:c>
-      <x:c r="W3" s="33" t="str">
+      <x:c r="X3" s="33" t="str">
         <x:v>title_skeleton</x:v>
       </x:c>
-      <x:c r="X3" s="33" t="str">
+      <x:c r="Y3" s="33" t="str">
         <x:v>source_files</x:v>
       </x:c>
-      <x:c r="Y3" s="33" t="str">
+      <x:c r="Z3" s="33" t="str">
         <x:v>duplicate_status</x:v>
       </x:c>
-      <x:c r="Z3" s="33" t="str">
+      <x:c r="AA3" t="str">
         <x:v>data_note</x:v>
       </x:c>
-      <x:c r="AA3" t="str">
+      <x:c r="AB3" t="str">
         <x:v>score</x:v>
       </x:c>
     </x:row>
@@ -40769,73 +40773,76 @@
         <x:v>当日热点强度与历史验证度最高，且适合熟龄账号</x:v>
       </x:c>
       <x:c r="D4" s="20" t="str">
+        <x:v>人到晚年才明白：儿女真正能托底的，不是钱，而是这份担当</x:v>
+      </x:c>
+      <x:c r="E4" s="20" t="str">
         <x:v>T0494</x:v>
-      </x:c>
-      <x:c r="E4" s="20" t="str">
-        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="F4" s="34" t="str">
         <x:v>2026-09-22</x:v>
       </x:c>
-      <x:c r="G4" s="34" t="n">
-        <x:v>1</x:v>
+      <x:c r="G4" s="34" t="str">
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="H4" s="20" t="n">
-        <x:v>100000</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="20" t="n">
         <x:v>100000</x:v>
       </x:c>
-      <x:c r="J4" s="20" t="str">
+      <x:c r="J4" s="20" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="K4" s="20" t="str">
         <x:v>韩粱最终娶了董氏，她还为韩粱生下一个儿子，在韩粱死后，是林锦岐出手护住了他的妻儿</x:v>
       </x:c>
-      <x:c r="K4" s="20" t="str"/>
-      <x:c r="L4" s="20" t="str">
+      <x:c r="L4" s="20" t="str"/>
+      <x:c r="M4" s="20" t="str">
         <x:v>2026-09-22 14:00:07</x:v>
       </x:c>
-      <x:c r="M4" s="20" t="str">
+      <x:c r="N4" s="20" t="str">
         <x:v>https://mp.weixin.qq.com/s?__biz=MzYyMzE4MTM0Nw==&amp;mid=2247485348&amp;idx=1&amp;sn=d1ea5b0ff9146580027eca40b0b06b06</x:v>
       </x:c>
-      <x:c r="N4" s="20" t="str">
+      <x:c r="O4" s="20" t="str">
         <x:v>https://mmbiz.qpic.cn/mmbiz_jpg/ic0nDxsIalVJhKxTfy3YXbZVNYl24JY9onoxJtFtmQl6UvUhjzZalKjY1Pg4gic83tRE1lG2iagrusZFvj7aiaiaw5ibdoF2h0DQbyxDLLXVL0H2I/0?wx_fmt=jpeg</x:v>
       </x:c>
-      <x:c r="O4" s="20" t="str">
-        <x:v>50岁以后</x:v>
-      </x:c>
       <x:c r="P4" s="20" t="str">
+        <x:v>50岁以后</x:v>
+      </x:c>
+      <x:c r="Q4" s="20" t="str">
         <x:v>代际关系与家庭边界</x:v>
       </x:c>
-      <x:c r="Q4" s="20" t="str">
+      <x:c r="R4" s="20" t="str">
         <x:v>子女关系与家庭边界</x:v>
       </x:c>
-      <x:c r="R4" s="20" t="n">
+      <x:c r="S4" s="20" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="S4" s="20" t="str">
+      <x:c r="T4" s="20" t="str">
         <x:v>50岁以上</x:v>
       </x:c>
-      <x:c r="T4" s="20" t="str">
+      <x:c r="U4" s="20" t="str">
         <x:v>男性偏强</x:v>
       </x:c>
-      <x:c r="U4" s="20" t="str">
-        <x:v>好奇/实用</x:v>
-      </x:c>
       <x:c r="V4" s="20" t="str">
+        <x:v>好奇/实用</x:v>
+      </x:c>
+      <x:c r="W4" s="20" t="str">
         <x:v>关系处理</x:v>
       </x:c>
-      <x:c r="W4" s="20" t="str">
+      <x:c r="X4" s="20" t="str">
         <x:v>事件切入型</x:v>
       </x:c>
-      <x:c r="X4" s="20" t="str">
+      <x:c r="Y4" s="20" t="str">
         <x:v>921432_微信24h热文榜_20260922.xlsx</x:v>
       </x:c>
-      <x:c r="Y4" s="20" t="str">
-        <x:v>唯一</x:v>
-      </x:c>
       <x:c r="Z4" s="20" t="str">
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="AA4" t="str">
         <x:v>引用历史老年主题分类或规则映射</x:v>
       </x:c>
-      <x:c r="AA4" t="n">
+      <x:c r="AB4" t="n">
         <x:v>23.5</x:v>
       </x:c>
     </x:row>
@@ -40850,80 +40857,83 @@
         <x:v>具备熟龄改造空间，作为今日备选</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
+        <x:v>身体这处毛发变白，真的暗示活不长吗？50岁后先别急着下结论</x:v>
+      </x:c>
+      <x:c r="E5" s="20" t="str">
         <x:v>T0508</x:v>
-      </x:c>
-      <x:c r="E5" s="20" t="str">
-        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="F5" s="34" t="str">
         <x:v>2026-09-22</x:v>
       </x:c>
-      <x:c r="G5" s="34" t="n">
-        <x:v>1</x:v>
+      <x:c r="G5" s="34" t="str">
+        <x:v>2026-09-22</x:v>
       </x:c>
       <x:c r="H5" s="20" t="n">
-        <x:v>56000</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="20" t="n">
         <x:v>56000</x:v>
       </x:c>
-      <x:c r="J5" s="20" t="str">
+      <x:c r="J5" s="20" t="n">
+        <x:v>56000</x:v>
+      </x:c>
+      <x:c r="K5" s="20" t="str">
         <x:v>身体这处毛发变白，暗示活得不长？看看你白了没有</x:v>
       </x:c>
-      <x:c r="K5" s="20" t="str"/>
-      <x:c r="L5" s="20" t="str">
+      <x:c r="L5" s="20" t="str"/>
+      <x:c r="M5" s="20" t="str">
         <x:v>2026-09-22 14:00:07</x:v>
       </x:c>
-      <x:c r="M5" s="20" t="str">
+      <x:c r="N5" s="20" t="str">
         <x:v>https://mp.weixin.qq.com/s?__biz=MzI4MDIxOTQxOA==&amp;mid=2247498461&amp;idx=1&amp;sn=784aa4654fd95aec8399a5226bbbff34</x:v>
       </x:c>
-      <x:c r="N5" s="20" t="str">
+      <x:c r="O5" s="20" t="str">
         <x:v>https://mmbiz.qpic.cn/mmbiz_jpg/ByeGEkGAjyhbeJiaTjunc24Nb6GyDAamraMFrzMS8CvBffeyBPrVefuO2hSeD7EbB4oVe6dULGvDHCbklDhdDcd955Wq3qB9bzicsItibOQYEM/0?wx_fmt=jpeg</x:v>
       </x:c>
-      <x:c r="O5" s="20" t="str">
-        <x:v>50岁以后</x:v>
-      </x:c>
       <x:c r="P5" s="20" t="str">
+        <x:v>50岁以后</x:v>
+      </x:c>
+      <x:c r="Q5" s="20" t="str">
         <x:v>健康饮食与运动</x:v>
       </x:c>
-      <x:c r="Q5" s="20" t="str">
+      <x:c r="R5" s="20" t="str">
         <x:v>50岁后的健康管理</x:v>
       </x:c>
-      <x:c r="R5" s="20" t="n">
+      <x:c r="S5" s="20" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="S5" s="20" t="str">
+      <x:c r="T5" s="20" t="str">
         <x:v>50岁以上</x:v>
       </x:c>
-      <x:c r="T5" s="20" t="str">
-        <x:v>通用</x:v>
-      </x:c>
       <x:c r="U5" s="20" t="str">
-        <x:v>好奇/实用</x:v>
+        <x:v>通用</x:v>
       </x:c>
       <x:c r="V5" s="20" t="str">
+        <x:v>好奇/实用</x:v>
+      </x:c>
+      <x:c r="W5" s="20" t="str">
         <x:v>改善身体</x:v>
       </x:c>
-      <x:c r="W5" s="20" t="str">
+      <x:c r="X5" s="20" t="str">
         <x:v>问题型</x:v>
       </x:c>
-      <x:c r="X5" s="20" t="str">
+      <x:c r="Y5" s="20" t="str">
         <x:v>921432_微信24h热文榜_20260922.xlsx</x:v>
       </x:c>
-      <x:c r="Y5" s="20" t="str">
-        <x:v>唯一</x:v>
-      </x:c>
       <x:c r="Z5" s="20" t="str">
+        <x:v>唯一</x:v>
+      </x:c>
+      <x:c r="AA5" t="str">
         <x:v>引用历史老年主题分类或规则映射</x:v>
       </x:c>
-      <x:c r="AA5" t="n">
+      <x:c r="AB5" t="n">
         <x:v>19.1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8095aeb112a4e25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74503f9bb4f849bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>